<commit_message>
feat: Unify dashboard logo to mountain mark + add sales targets and articles
- Replace Activity icon with mountain mark SVG across dashboard (Auth, AdminRoute, Dashboard)
- Add 11 AI contract development companies to sales target list
- Add Zenn/Qiita educational articles on LLM observability and RAG tracing

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sales-target-list.xlsx
+++ b/docs/sales-target-list.xlsx
@@ -62,7 +62,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -84,11 +84,17 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -103,6 +109,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -470,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1468,6 +1477,523 @@
       <c r="I21" t="inlineStr">
         <is>
           <t>SaaS型。AIエージェント技術でテスト自動化を行い、内部でLLMを活用。テスト実行時のAI判断精度・コスト・パフォーマンスのトレースにFujiTraceが有用。クライアント企業のCI/CDパイプラインに組み込まれるため監視ニーズが高い。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>株式会社知能情報システム</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>AI受託開発（LLM/エージェント特化）</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>https://www.iknowledge.co.jp/</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>LLM活用受託開発（LangGraph/CrewAI）</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>LLMとLangGraph・CrewAI等の最新フレームワークを活用し、研究開発業務の自動化を受託開発。エージェント開発が主力</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>不明（小規模推定）</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>東京都</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>受託チャネル型。LLMエージェント開発が主力業務のため、トレース・デバッグ需要が直接的。受託案件ごとにFujiTraceを「運用監視キット」としてセット納品可能。エージェント開発=マルチステップLLM呼び出しのため、オブザバビリティの価値が最大化される。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>アーガイル株式会社</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>AI受託開発（ChatGPT API連携特化）</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>https://chatgpt-api-developper.argyle.jp/</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>生成AIシステム受託開発（AIエージェント・チャットボット・画像生成）</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>ChatGPT・Gemini等のLLM API連携によるチャットボット・AIエージェント・画像生成システムの受託開発を専門に提供</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>不明（小規模推定）</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>東京都</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>受託チャネル型。LLM API呼び出しが業務の中核。クライアント企業に納品するチャットボット・AIエージェントのトレース・コスト管理にFujiTraceが直結。複数案件へのレバレッジが効く。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>株式会社ProFab</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>AI受託開発（Dify活用ローコード）</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>Dify活用ローコードAI実装受託</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>ローコードAI開発ツール「Dify」を活用し短期間でのAI実装を受託。経営コンサルティング背景を持つチームが導入を支援</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>不明（小規模推定）</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>東京都</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>受託チャネル型。Difyを活用してLLMアプリを量産する体制。案件ごとにFujiTraceを組み込めば、クライアント側でのLLM利用量・品質監視を標準提供でき、納品物の付加価値向上+FujiTraceの販路拡大。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>株式会社ニューラルオプト</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>AI受託開発（生成AIコンサル+PoC）</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>https://neural-opt.com/</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>生成AIコンサルティング / PoC開発</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>2024年設立。課題起点のAIコンサル×PoC特化。ChatGPT開発経験・データサイエンスを活かしたコスト効率の高いソリューション提供</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>2024年</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>不明（小規模推定）</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>東京都</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>受託チャネル型。新興で意思決定が速い。PoC段階でのLLMトレース可視化はクライアントへの説得材料になるため、FujiTraceをPoC標準ツールとして採用する動機が強い。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>DAI Labs株式会社</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>AI受託開発（スタートアップ・中小向け）</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>生成AI/LLM活用受託開発</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>生成AI・LLM活用に注力。スタートアップや中小企業からの初期相談に柔軟に対応し、コストを抑えた段階的な開発に対応</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>不明（小規模推定）</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>東京都</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>受託チャネル型。小規模案件を多数抱える構造。案件ごとにFujiTraceを導入すれば、クライアント側のLLMコスト可視化・品質管理を低コストで提供でき、DAI Labsの差別化要因にもなる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>株式会社エクスプラザ</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>AI受託開発（RAG/エージェント）</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>https://and-and.co.jp/</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>RAG構築・AIエージェント受託開発</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>生成AI活用で企業の成長を支援。RAG構築・精度改善、文書要約ツール、マルチモーダルシステム、AIエージェント開発。直近1年でPoC30件以上、本開発15件以上の実績</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>不明（小規模推定）</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>東京都</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>受託チャネル型。RAG+エージェント開発がまさにオブザバビリティの需要層。RAGパイプライン（検索→生成）のトレースは品質改善の要。PoC・本開発合わせて45件+の実績があり、各案件にFujiTraceを標準導入すれば大きなレバレッジ。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>株式会社AVILEN</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>AI受託開発（コンサル+開発一貫）</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>https://avilen.co.jp/</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>AI受託開発 / AIコンサルティング / AI人材育成</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>東大発ベンチャー。800社以上の支援実績。AIコンサルタントが戦略立案から開発まで一貫対応。自然言語処理・画像解析等の最先端アルゴリズムを自社開発</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>2018年</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>不明（中規模推定）</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>東京都</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>受託チャネル型。800社+という圧倒的な支援実績。LLM案件も増加中で、クライアント企業へのFujiTrace標準導入が実現すれば最大のレバレッジ。規模感からパートナーシップ交渉のハードルはやや高いが、リターンも大きい。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>株式会社Laboro.AI</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>AI受託開発（完全カスタム）</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>https://laboro.ai/</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>カスタムAIソリューション受託開発</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>2016年創業。完全受託型でAI開発を行い、約70%の高いプロジェクト継続率。SaaS制約なしの高度なカスタマイズが強み。幅広い産業のトップ企業向けに提供</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>2016年</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>不明（中規模推定）</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>東京都</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>受託チャネル型。継続率70%＝長期案件が多く、運用フェーズでのLLMモニタリング需要が高い。完全カスタム開発のためFujiTraceを案件ごとに組み込む柔軟性がある。LLM案件の比率確認が必要。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>株式会社ギブリー</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>AI受託開発 / 自社SaaS</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>https://givery.co.jp/</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>法人GAI / Track / DECA / MANA</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>2009年設立。生成AI活用に特化し600社+支援実績。18ヶ国以上のスペシャリストによるグローバルチーム。法人GAI（¥980/人/月）等の自社プロダクトも保有</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>2009年</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>不明（中規模推定）</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>東京都</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>受託+SaaSハイブリッド型。法人GAIは企業がLLMを利用するPFで、利用企業側のトレース・コスト管理にFujiTraceが有用。600社+の支援実績からリーチが広い。自社SaaS寄りだが受託案件もあり。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>株式会社リベルクラフト</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>AI受託開発（データ分析+内製化支援）</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>https://liber-craft.co.jp/</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>データ分析・AI/ML受託開発 / 内製化支援</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>データ分析とAI・機械学習で顧客課題を解決。人材育成による内製化支援も実施。クライアント企業のAI自走を支援するモデル</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>不明（小規模推定）</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>東京都</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>受託チャネル型。内製化支援モデルのため、クライアント企業が自社でLLMを運用するフェーズでFujiTraceが必要になる。「内製化後の監視ツール」としてセット提案可能。LLM案件の有無確認が必要。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>木村情報技術株式会社</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>AI受託開発（製薬業界特化）</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>https://www.kimura-it.co.jp/</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>製薬業界向けAIチャットボット</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>製薬業界向けAIチャットボットで導入実績No.1。70名の専門チームで業界特有ニーズに対応。製薬業界のコンプライアンス要件を熟知</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>不明</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>約70名</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>佐賀県</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>受託チャネル型。製薬業界はコンプライアンス要件が極めて厳しく、LLM出力のトレース・監査ログは必須要件。「薬事規制対応のためのLLMトレース」という切り口でFujiTraceが刺さる可能性が高い。業界No.1の導入実績からレバレッジも大きい。</t>
         </is>
       </c>
     </row>

</xml_diff>